<commit_message>
save confirmation screen — separate screen outside tabs, read-only form detail, only deletes saved forms
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JUN" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEP" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUG" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAY" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOV" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,9 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="D-MMM"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="D-MMM"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -70,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -79,7 +80,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -195,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J5" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J10" headerRowCount="1">
   <autoFilter ref="A3:J5"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -234,6 +236,44 @@
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="InKind_AUG" displayName="InKind_AUG" ref="A3:J4" headerRowCount="1">
+  <autoFilter ref="A3:J4"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="DATE"/>
+    <tableColumn id="2" name="SOURCE"/>
+    <tableColumn id="3" name="PERISHABLE"/>
+    <tableColumn id="4" name="NON-PERISHABLE"/>
+    <tableColumn id="5" name="MEAT"/>
+    <tableColumn id="6" name="DAIRY"/>
+    <tableColumn id="7" name="EGGS"/>
+    <tableColumn id="8" name="PRODUCE"/>
+    <tableColumn id="9" name="MONTHLY TOTAL"/>
+    <tableColumn id="10" name="YTD"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InKind_MAY" displayName="InKind_MAY" ref="A3:J11" headerRowCount="1">
+  <autoFilter ref="A3:J11"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="DATE"/>
+    <tableColumn id="2" name="SOURCE"/>
+    <tableColumn id="3" name="PERISHABLE"/>
+    <tableColumn id="4" name="NON-PERISHABLE"/>
+    <tableColumn id="5" name="MEAT"/>
+    <tableColumn id="6" name="DAIRY"/>
+    <tableColumn id="7" name="EGGS"/>
+    <tableColumn id="8" name="PRODUCE"/>
+    <tableColumn id="9" name="MONTHLY TOTAL"/>
+    <tableColumn id="10" name="YTD"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="InKind_NOV" displayName="InKind_NOV" ref="A3:J4" headerRowCount="1">
   <autoFilter ref="A3:J4"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -654,7 +694,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>44771</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -803,7 +843,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>45343</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -819,7 +859,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>44614</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -841,7 +881,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>44251</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -876,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -990,7 +1030,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>44739</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1027,6 +1067,20 @@
         <v>72</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>45828</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MacBook-Air</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -1158,7 +1212,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>44828</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1310,7 +1364,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>44435</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1326,6 +1380,356 @@
       </c>
       <c r="I4" t="n">
         <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS: Enter as per weigh-in logs by scale in WH. Always enter value under perishable or non-perishable AND under appropriate category i.e. "produce" or "meat".</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTAL</t>
+        </is>
+      </c>
+      <c r="C2">
+        <f>SUM(InKind_MAY[PERISHABLE])</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>SUM(InKind_MAY[NON-PERISHABLE])</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>SUM(InKind_MAY[MEAT])</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>SUM(InKind_MAY[DAIRY])</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUM(InKind_MAY[EGGS])</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUM(InKind_MAY[PRODUCE])</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUM(InKind_MAY[MONTHLY TOTAL])</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUM(InKind_MAY[YTD])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>PERISHABLE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>NON-PERISHABLE</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>MEAT</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>DAIRY</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>EGGS</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTAL</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>45075</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>44701</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>44336</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>43614</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>43232</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>42153</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>42152</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>41406</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS: Enter as per weigh-in logs by scale in WH. Always enter value under perishable or non-perishable AND under appropriate category i.e. "produce" or "meat".</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTAL</t>
+        </is>
+      </c>
+      <c r="C2">
+        <f>SUM(InKind_NOV[PERISHABLE])</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>SUM(InKind_NOV[NON-PERISHABLE])</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>SUM(InKind_NOV[MEAT])</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>SUM(InKind_NOV[DAIRY])</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUM(InKind_NOV[EGGS])</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUM(InKind_NOV[PRODUCE])</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUM(InKind_NOV[MONTHLY TOTAL])</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUM(InKind_NOV[YTD])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>PERISHABLE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>NON-PERISHABLE</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>MEAT</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>DAIRY</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>EGGS</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCE</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTAL</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>43773</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix deleteForm race condition — use write queue
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J10" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J9" headerRowCount="1">
   <autoFilter ref="A3:J5"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -916,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1080,7 +1080,6 @@
     <row r="7"/>
     <row r="8"/>
     <row r="9"/>
-    <row r="10"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
add analyzing hint message in Review screen
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J9" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J10" headerRowCount="1">
   <autoFilter ref="A3:J5"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InKind_MAY" displayName="InKind_MAY" ref="A3:J11" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InKind_MAY" displayName="InKind_MAY" ref="A3:J12" headerRowCount="1">
   <autoFilter ref="A3:J11"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -916,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1077,9 +1077,61 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Yu66u</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>856</v>
+      </c>
+      <c r="I7" t="n">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>320</v>
+      </c>
+      <c r="D8" t="n">
+        <v>160</v>
+      </c>
+      <c r="F8" t="n">
+        <v>320</v>
+      </c>
+      <c r="I8" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>360</v>
+      </c>
+      <c r="D9" t="n">
+        <v>160</v>
+      </c>
+      <c r="F9" t="n">
+        <v>360</v>
+      </c>
+      <c r="I9" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="10"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -1398,7 +1450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1513,7 +1565,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>45075</v>
+        <v>41406</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1523,7 +1575,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>44701</v>
+        <v>45075</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1533,7 +1585,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>44336</v>
+        <v>44701</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1543,7 +1595,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>43614</v>
+        <v>44336</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1553,7 +1605,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>43232</v>
+        <v>43614</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1563,7 +1615,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>42153</v>
+        <v>43232</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1573,7 +1625,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>42152</v>
+        <v>42153</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1583,9 +1635,19 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
+        <v>42152</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
         <v>41406</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Port BIC</t>
         </is>

</xml_diff>

<commit_message>
fix find_insert_row — correctly handle blank date rows in date ordering
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -153,8 +153,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J4" headerRowCount="1">
-  <autoFilter ref="A3:J4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J6" headerRowCount="1">
+  <autoFilter ref="A3:J6"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
     <tableColumn id="2" name="SOURCE"/>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -577,6 +577,58 @@
       <c r="A4" s="4" t="n">
         <v>46191</v>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SDE</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Loblaws</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" t="n">
+        <v>110</v>
+      </c>
+      <c r="I5" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LobLaws</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="n">
+        <v>110</v>
+      </c>
+      <c r="I6" t="n">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
fix landscape photo rotation using EXIF orientation data
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="D-MMM"/>
+    <numFmt numFmtId="164" formatCode="D-MMM"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -75,7 +75,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -153,8 +154,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J6" headerRowCount="1">
-  <autoFilter ref="A3:J6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J19" headerRowCount="1">
+  <autoFilter ref="A3:J12"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
     <tableColumn id="2" name="SOURCE"/>
@@ -460,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -574,60 +575,250 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>46191</v>
+      <c r="A4" s="5" t="n">
+        <v>46180</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SDE</t>
+          <t>Timmies</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
-      </c>
-      <c r="D4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I4" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" t="n">
+        <v>45</v>
+      </c>
+      <c r="I5" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I6" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Food Basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" t="n">
+        <v>80</v>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>100</v>
       </c>
-      <c r="I4" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Anon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>46180</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Loblaws</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
-      <c r="D5" t="n">
-        <v>110</v>
-      </c>
-      <c r="I5" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>LobLaws</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
-      <c r="D6" t="n">
-        <v>110</v>
-      </c>
-      <c r="I6" t="n">
-        <v>140</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>45</v>
+      </c>
+      <c r="F13" t="n">
+        <v>45</v>
+      </c>
+      <c r="I13" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Food Basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>80</v>
+      </c>
+      <c r="E15" t="n">
+        <v>80</v>
+      </c>
+      <c r="I15" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sobeys</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>102</v>
+      </c>
+      <c r="H16" t="n">
+        <v>102</v>
+      </c>
+      <c r="I16" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Central United</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>20</v>
+      </c>
+      <c r="I19" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added table overlay, updates to form details preview
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="D-MMM"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -154,7 +153,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J19" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J20" headerRowCount="1">
   <autoFilter ref="A3:J12"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -461,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -821,6 +820,7 @@
         <v>20</v>
       </c>
     </row>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
parallel OCR and preview crop, loading placeholder in form detail
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="D-MMM"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -153,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J20" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J24" headerRowCount="1">
   <autoFilter ref="A3:J12"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -460,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -575,252 +576,331 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>46180</v>
+        <v>46178</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Timmies</t>
+          <t>No Frills</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>45</v>
-      </c>
-      <c r="F4" t="n">
-        <v>45</v>
+        <v>80</v>
+      </c>
+      <c r="E4" t="n">
+        <v>80</v>
       </c>
       <c r="I4" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46180</v>
+        <v>46177</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Timmies</t>
+          <t>Sobey's</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>45</v>
-      </c>
-      <c r="F5" t="n">
-        <v>45</v>
+        <v>102</v>
+      </c>
+      <c r="H5" t="n">
+        <v>102</v>
       </c>
       <c r="I5" t="n">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46180</v>
+        <v>46176</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Timmies</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>45</v>
-      </c>
-      <c r="F6" t="n">
-        <v>45</v>
-      </c>
-      <c r="I6" t="n">
-        <v>45</v>
+          <t>Central United</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46179</v>
+        <v>46175</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Food Basics</t>
-        </is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>46178</v>
+        <v>46174</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>No Frills</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>80</v>
-      </c>
-      <c r="E8" t="n">
-        <v>80</v>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>20</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vale</t>
+          <t>Timmies</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>100</v>
+        <v>45</v>
+      </c>
+      <c r="F9" t="n">
+        <v>45</v>
       </c>
       <c r="I9" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>46174</v>
+        <v>46180</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Port BIC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>20</v>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>45</v>
+      </c>
+      <c r="F10" t="n">
+        <v>45</v>
       </c>
       <c r="I10" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46182</v>
+        <v>46180</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Anon</t>
-        </is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" t="n">
+        <v>45</v>
+      </c>
+      <c r="I11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>46181</v>
+        <v>46179</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SDM</t>
+          <t>Food Basics</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>46180</v>
+        <v>46178</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Timmies</t>
+          <t>No Frills</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>45</v>
-      </c>
-      <c r="F13" t="n">
-        <v>45</v>
+        <v>80</v>
+      </c>
+      <c r="E13" t="n">
+        <v>80</v>
       </c>
       <c r="I13" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>46179</v>
+        <v>46175</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Food Basics</t>
-        </is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>100</v>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46178</v>
+        <v>46174</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>No Frills</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>80</v>
-      </c>
-      <c r="E15" t="n">
-        <v>80</v>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>20</v>
       </c>
       <c r="I15" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sobeys</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>102</v>
-      </c>
-      <c r="H16" t="n">
-        <v>102</v>
-      </c>
-      <c r="I16" t="n">
-        <v>102</v>
+          <t>Anon</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Central United</t>
+          <t>SDM</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vale</t>
+          <t>Timmies</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>100</v>
+        <v>45</v>
+      </c>
+      <c r="F18" t="n">
+        <v>45</v>
       </c>
       <c r="I18" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Food Basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>80</v>
+      </c>
+      <c r="E20" t="n">
+        <v>80</v>
+      </c>
+      <c r="I20" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sobeys</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>102</v>
+      </c>
+      <c r="H21" t="n">
+        <v>102</v>
+      </c>
+      <c r="I21" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Central United</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
         <v>46174</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Port BIC</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D24" t="n">
         <v>20</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I24" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="20"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
focus button label, preview loading hint, parallel OCR and preview generation
</commit_message>
<xml_diff>
--- a/server/data/Port Cares In 2026.xlsx
+++ b/server/data/Port Cares In 2026.xlsx
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J24" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InKind_JUN" displayName="InKind_JUN" ref="A3:J34" headerRowCount="1">
   <autoFilter ref="A3:J12"/>
   <tableColumns count="10">
     <tableColumn id="1" name="DATE"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -576,149 +576,143 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>46178</v>
+        <v>46177</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>No Frills</t>
+          <t>Sobeys</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>80</v>
-      </c>
-      <c r="E4" t="n">
-        <v>80</v>
+        <v>102</v>
+      </c>
+      <c r="H4" t="n">
+        <v>102</v>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46177</v>
+        <v>46176</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sobey's</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>102</v>
-      </c>
-      <c r="H5" t="n">
-        <v>102</v>
-      </c>
-      <c r="I5" t="n">
-        <v>102</v>
+          <t>Central United</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46176</v>
+        <v>46175</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Central United</t>
-        </is>
+          <t>Yale</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46175</v>
+        <v>46174</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vale</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>100</v>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
       </c>
       <c r="I7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Port BIC</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>20</v>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" t="n">
+        <v>80</v>
       </c>
       <c r="I8" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46180</v>
+        <v>46177</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Timmies</t>
+          <t>Sobey's</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>45</v>
-      </c>
-      <c r="F9" t="n">
-        <v>45</v>
+        <v>102</v>
+      </c>
+      <c r="H9" t="n">
+        <v>102</v>
       </c>
       <c r="I9" t="n">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>46180</v>
+        <v>46176</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timmies</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>45</v>
-      </c>
-      <c r="F10" t="n">
-        <v>45</v>
-      </c>
-      <c r="I10" t="n">
-        <v>45</v>
+          <t>Central United</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46180</v>
+        <v>46175</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Timmies</t>
+          <t>Vale</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>45</v>
-      </c>
-      <c r="F11" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="I11" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>46179</v>
+        <v>46174</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Food Basics</t>
-        </is>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -742,163 +736,326 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vale</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>100</v>
-      </c>
-      <c r="I14" t="n">
-        <v>100</v>
+          <t>Food Basics</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46174</v>
+        <v>46180</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Port BIC</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>20</v>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>45</v>
+      </c>
+      <c r="F15" t="n">
+        <v>45</v>
       </c>
       <c r="I15" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>46182</v>
+        <v>46180</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Anon</t>
-        </is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>45</v>
+      </c>
+      <c r="F16" t="n">
+        <v>45</v>
+      </c>
+      <c r="I16" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46181</v>
+        <v>46180</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SDM</t>
-        </is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" t="n">
+        <v>45</v>
+      </c>
+      <c r="I17" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>46180</v>
+        <v>46179</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Timmies</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>45</v>
-      </c>
-      <c r="F18" t="n">
-        <v>45</v>
-      </c>
-      <c r="I18" t="n">
-        <v>45</v>
+          <t>Food Basics</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>46179</v>
+        <v>46178</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Food Basics</t>
-        </is>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E19" t="n">
+        <v>80</v>
+      </c>
+      <c r="I19" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>46178</v>
+        <v>46175</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>No Frills</t>
+          <t>Vale</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>80</v>
-      </c>
-      <c r="E20" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I20" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>46177</v>
+        <v>46174</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sobeys</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>102</v>
-      </c>
-      <c r="H21" t="n">
-        <v>102</v>
+          <t>Port BIC</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>20</v>
       </c>
       <c r="I21" t="n">
-        <v>102</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Central United</t>
-        </is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" t="n">
+        <v>45</v>
+      </c>
+      <c r="I22" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>46175</v>
+        <v>46181</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Vale</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>100</v>
-      </c>
-      <c r="I23" t="n">
-        <v>100</v>
+          <t>SDM</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Anon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Timmies</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>45</v>
+      </c>
+      <c r="F26" t="n">
+        <v>45</v>
+      </c>
+      <c r="I26" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Food Basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>No Frills</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>80</v>
+      </c>
+      <c r="E28" t="n">
+        <v>80</v>
+      </c>
+      <c r="I28" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sobeys</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>102</v>
+      </c>
+      <c r="H29" t="n">
+        <v>102</v>
+      </c>
+      <c r="I29" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Central United</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>100</v>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
         <v>46174</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Port BIC</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D32" t="n">
         <v>20</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I32" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Anon</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Archies</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>115</v>
+      </c>
+      <c r="D34" t="n">
+        <v>20</v>
+      </c>
+      <c r="E34" t="n">
+        <v>19</v>
+      </c>
+      <c r="F34" t="n">
+        <v>45</v>
+      </c>
+      <c r="H34" t="n">
+        <v>30</v>
+      </c>
+      <c r="I34" t="n">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>